<commit_message>
Dados atualizados via Robô: Sun Apr  5 04:03:29 UTC 2026
</commit_message>
<xml_diff>
--- a/sipii_caixa_20260405.xlsx
+++ b/sipii_caixa_20260405.xlsx
@@ -14,9 +14,9 @@
     <sheet name="RENDA FIXA CURTO PRAZO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="MULTIMERCADO" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="CAMBIAL" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="AÇÕES" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FUNDO DE ÍNDICE" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FUNDOS MÚTUOS DE PRIVATIZAÇÃO" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ACOES" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FUNDO DE INDICE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FUNDOS MUTUOS DE PRIVATIZACAO" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +450,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -485,12 +485,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -550,6 +555,11 @@
           <t>426,362</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/esimples-renda-fixa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -607,6 +617,11 @@
           <t>6.533,853</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/fic-facil-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -664,6 +679,11 @@
           <t>800,750</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/fic-movimentacoes-automaticas-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -721,6 +741,11 @@
           <t>10,743</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-geracao-jovem-cred-priv-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -778,6 +803,11 @@
           <t>582,057</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-ideal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -835,6 +865,11 @@
           <t>1.427,057</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-exclusivo-func-rf-credito-privado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -892,6 +927,11 @@
           <t>28,637</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-capital-ind-precos-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -949,6 +989,11 @@
           <t>115,072</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-personal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1006,6 +1051,11 @@
           <t>100,344</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/master-plus-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1063,6 +1113,11 @@
           <t>121,555</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-absoluto-pre-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1120,6 +1175,11 @@
           <t>58,849</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-efundo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1177,6 +1237,11 @@
           <t>65,791</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-soberano-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1234,6 +1299,11 @@
           <t>39,323</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-empreender-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1291,6 +1361,11 @@
           <t>27,651</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-classico-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1348,6 +1423,11 @@
           <t>86,249</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-foco-ind-precos-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1405,6 +1485,11 @@
           <t>1,893</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-desenvolver-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1462,6 +1547,11 @@
           <t>128,171</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-objetivo-pre-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1519,6 +1609,11 @@
           <t>1.445,497</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-oab-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1576,6 +1671,11 @@
           <t>13,796</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-ideal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1633,6 +1733,11 @@
           <t>2.137,571</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-executivo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1690,6 +1795,11 @@
           <t>66,296</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-performance-imab-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1747,6 +1857,11 @@
           <t>954,612</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-fifinvestidor-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1804,6 +1919,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-absolute-creta-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1861,6 +1981,11 @@
           <t>194,710</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-plus-quali-rf-credi-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1918,6 +2043,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-expert-sulamerica-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1975,6 +2105,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-arx-ipca-deb-incentivadas-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2032,6 +2167,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-vox-desenv-sustentavel-is-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2089,6 +2229,11 @@
           <t>34,940</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/inflacao-private-2027-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2146,6 +2291,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-rb-asset-cdi-deb-incentivadas-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2203,6 +2353,11 @@
           <t>2.894,171</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-expertise-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2260,6 +2415,11 @@
           <t>866,715</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/qualificado-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2317,6 +2477,11 @@
           <t>19,483</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-selecao-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2374,6 +2539,11 @@
           <t>133,651</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-renda-fixa-ativa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2431,6 +2601,11 @@
           <t>313,138</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/indexa-tesouro-selic-fic-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2488,6 +2663,11 @@
           <t>3.103,041</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-personal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2545,6 +2725,11 @@
           <t>125,908</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-supremo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2602,6 +2787,11 @@
           <t>149,794</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-unique-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2659,6 +2849,11 @@
           <t>2.398,591</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-especial-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2716,6 +2911,11 @@
           <t>14.155,221</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-maxi-renda-fixa-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2773,6 +2973,11 @@
           <t>531,259</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fidelidade-private-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2830,6 +3035,11 @@
           <t>1.293,248</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fidelidade-ii-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2887,6 +3097,11 @@
           <t>153,838</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-beta-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2944,6 +3159,11 @@
           <t>5.163,293</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-giro-imediato-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3001,6 +3221,11 @@
           <t>47,704</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-omega-ref-di-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3058,6 +3283,11 @@
           <t>2.048,258</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-pleno-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3115,6 +3345,11 @@
           <t>872,706</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-preferencial-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3172,6 +3407,11 @@
           <t>13.911,673</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-sigma-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3229,6 +3469,11 @@
           <t>9.604,168</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-rubi-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3286,6 +3531,11 @@
           <t>18.273,507</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-mega-rf-referenc-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3343,6 +3593,11 @@
           <t>10.092,191</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-top-private-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3400,6 +3655,11 @@
           <t>237,414</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-curto-prazo/fic-renda-fixa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3457,6 +3717,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-cred-priv-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3514,6 +3779,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-multigestor-global-equit-s/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3571,6 +3841,11 @@
           <t>2.039,830</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-bolsa-americana-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3628,6 +3903,11 @@
           <t>21,113</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-juros-e-moedas-mm-plus/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3685,6 +3965,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-funcionarios-estrategia-livre-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3742,6 +4027,11 @@
           <t>540,034</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/multimercado-rv-30/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3799,6 +4089,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-estrategia-livre-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3856,6 +4151,11 @@
           <t>8,878</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-short-dolar-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3913,6 +4213,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-long-short/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3970,6 +4275,11 @@
           <t>2,907</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4027,6 +4337,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4084,6 +4399,11 @@
           <t>2,386</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-euro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4141,6 +4461,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-estrategico-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4198,6 +4523,11 @@
           <t>501,310</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-ouro-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4255,6 +4585,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-mult-strategia-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4312,6 +4647,11 @@
           <t>37,650</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-hedge-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4369,6 +4709,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/hashdex-nasdaq-crypto-index-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4426,6 +4771,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/capital-protegido-ciclico-iii-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4483,6 +4833,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/capital-protegido-ibovespa-ciclico-i-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4540,6 +4895,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fim-capital-protegido-ciclico-ii/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4597,6 +4957,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-cesta-agro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4654,6 +5019,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-expert-spx-nimitz-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4711,6 +5081,11 @@
           <t>891,384</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-alocacao-macro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4768,6 +5143,11 @@
           <t>799,440</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-juros-e-moedas-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4825,6 +5205,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-caixa-expert-btg-pactual-x10-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4882,6 +5267,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-expert-pimco-income-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4939,6 +5329,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/expert-giant-zarathustra-fic-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4996,11 +5391,16 @@
           <t>83,873</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/cambial/fic-indexa-dolar-cambial/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -5051,13 +5451,18 @@
       <c r="K81" t="inlineStr">
         <is>
           <t>302,922</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-dividendos/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5108,13 +5513,18 @@
       <c r="K82" t="inlineStr">
         <is>
           <t>11,995</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-efundos-ibovespa/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5165,13 +5575,18 @@
       <c r="K83" t="inlineStr">
         <is>
           <t>9,700</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/atena-fic-acoes-funcionarios-livre-quant/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5222,13 +5637,18 @@
       <c r="K84" t="inlineStr">
         <is>
           <t>299,253</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-bdr-nivel-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5279,13 +5699,18 @@
       <c r="K85" t="inlineStr">
         <is>
           <t>489,187</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-small-caps-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5336,13 +5761,18 @@
       <c r="K86" t="inlineStr">
         <is>
           <t>78,102</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-consumo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5393,13 +5823,18 @@
       <c r="K87" t="inlineStr">
         <is>
           <t>2,671</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-sustentabilidade-empresarial-ise-is/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5450,13 +5885,18 @@
       <c r="K88" t="inlineStr">
         <is>
           <t>65,705</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras-plus/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5507,13 +5947,18 @@
       <c r="K89" t="inlineStr">
         <is>
           <t>84,277</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-ibovespa/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5564,13 +6009,18 @@
       <c r="K90" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-multigestor/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5621,13 +6071,18 @@
       <c r="K91" t="inlineStr">
         <is>
           <t>147,465</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-construcao-civil/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5678,13 +6133,18 @@
       <c r="K92" t="inlineStr">
         <is>
           <t>127,311</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-infraestrutura/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5735,13 +6195,18 @@
       <c r="K93" t="inlineStr">
         <is>
           <t>47,594</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/atena-fic-acoes-livre-quant/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5792,13 +6257,18 @@
       <c r="K94" t="inlineStr">
         <is>
           <t>144,951</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras-presal/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5849,13 +6319,18 @@
       <c r="K95" t="inlineStr">
         <is>
           <t>50,924</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-banco-do-brasil-plus/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5906,13 +6381,18 @@
       <c r="K96" t="inlineStr">
         <is>
           <t>572,055</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-vale-do-rio-doce/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5963,13 +6443,18 @@
       <c r="K97" t="inlineStr">
         <is>
           <t>413,157</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-seguridade/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6020,13 +6505,18 @@
       <c r="K98" t="inlineStr">
         <is>
           <t>21,063</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-ibrx-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -6077,13 +6567,18 @@
       <c r="K99" t="inlineStr">
         <is>
           <t>31,693</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-setor-financeiro/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6134,13 +6629,18 @@
       <c r="K100" t="inlineStr">
         <is>
           <t>2,316</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-dividendos-quantitativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6191,13 +6691,18 @@
       <c r="K101" t="inlineStr">
         <is>
           <t>41,189</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-pibb-ibrx-50/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6248,13 +6753,18 @@
       <c r="K102" t="inlineStr">
         <is>
           <t>34,936</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-ibovespa-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6305,13 +6815,18 @@
       <c r="K103" t="inlineStr">
         <is>
           <t>764,909</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6362,13 +6877,18 @@
       <c r="K104" t="inlineStr">
         <is>
           <t>4,027</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-iagro/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6419,13 +6939,18 @@
       <c r="K105" t="inlineStr">
         <is>
           <t>4,875</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-compromisso-bdr-nivel-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6476,13 +7001,18 @@
       <c r="K106" t="inlineStr">
         <is>
           <t>20,989</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/seguridade-ii-acoes/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6533,13 +7063,18 @@
       <c r="K107" t="inlineStr">
         <is>
           <t>238,332</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-eletrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6590,13 +7125,18 @@
       <c r="K108" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-expert-verde-am-long-bias/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6647,13 +7187,18 @@
       <c r="K109" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/expert-claritas-valor-fic-acoes/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FUNDO DE ÍNDICE</t>
+          <t>FUNDO DE INDICE</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6704,13 +7249,18 @@
       <c r="K110" t="inlineStr">
         <is>
           <t>41,204</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundo-de-indice/etf-ibovespa-fundo-de-indice/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6761,13 +7311,18 @@
       <c r="K111" t="inlineStr">
         <is>
           <t>4,124</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-eletrobras-migracao/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6818,13 +7373,18 @@
       <c r="K112" t="inlineStr">
         <is>
           <t>1.421,679</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-eletrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6875,13 +7435,18 @@
       <c r="K113" t="inlineStr">
         <is>
           <t>596,906</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-iv/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6932,13 +7497,18 @@
       <c r="K114" t="inlineStr">
         <is>
           <t>666,240</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-ii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -6989,13 +7559,18 @@
       <c r="K115" t="inlineStr">
         <is>
           <t>116,972</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-cl-absoluto/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -7046,13 +7621,18 @@
       <c r="K116" t="inlineStr">
         <is>
           <t>10,204</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-migracao/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -7103,13 +7683,18 @@
       <c r="K117" t="inlineStr">
         <is>
           <t>491,324</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-ii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -7160,13 +7745,18 @@
       <c r="K118" t="inlineStr">
         <is>
           <t>388,337</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7217,6 +7807,11 @@
       <c r="K119" t="inlineStr">
         <is>
           <t>623,984</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-iii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -7231,7 +7826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7247,7 +7842,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -7262,12 +7857,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -7282,19 +7877,24 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7345,13 +7945,18 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>4,124</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-eletrobras-migracao/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7402,13 +8007,18 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>1.421,679</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-eletrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7459,13 +8069,18 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>596,906</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-iv/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7516,13 +8131,18 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>666,240</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-ii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7573,13 +8193,18 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>116,972</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-cl-absoluto/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7630,13 +8255,18 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>10,204</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-migracao/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7687,13 +8317,18 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>491,324</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-ii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7744,13 +8379,18 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>388,337</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-vale-rio-doce-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FUNDOS MÚTUOS DE PRIVATIZAÇÃO</t>
+          <t>FUNDOS MUTUOS DE PRIVATIZACAO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -7801,6 +8441,11 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>623,984</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundos-mutuos-de-privatizacao/fmpfgts-petrobras-iii/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -7815,7 +8460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7831,7 +8476,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -7846,12 +8491,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -7866,12 +8511,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -7931,6 +8581,11 @@
           <t>426,362</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/esimples-renda-fixa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7988,6 +8643,11 @@
           <t>6.533,853</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/fic-facil-rf-simples/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8043,6 +8703,11 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>800,750</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-simples/fic-movimentacoes-automaticas-rf-simples/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -8057,7 +8722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8073,7 +8738,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -8088,12 +8753,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -8108,12 +8773,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -8173,6 +8843,11 @@
           <t>10,743</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-geracao-jovem-cred-priv-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8230,6 +8905,11 @@
           <t>582,057</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-ideal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8287,6 +8967,11 @@
           <t>1.427,057</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-exclusivo-func-rf-credito-privado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8344,6 +9029,11 @@
           <t>28,637</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-capital-ind-precos-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8401,6 +9091,11 @@
           <t>115,072</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-personal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8458,6 +9153,11 @@
           <t>100,344</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/master-plus-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8515,6 +9215,11 @@
           <t>121,555</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-absoluto-pre-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8572,6 +9277,11 @@
           <t>58,849</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-efundo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8629,6 +9339,11 @@
           <t>65,791</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-soberano-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8686,6 +9401,11 @@
           <t>39,323</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-empreender-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8743,6 +9463,11 @@
           <t>27,651</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-classico-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8800,6 +9525,11 @@
           <t>86,249</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-foco-ind-precos-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8857,6 +9587,11 @@
           <t>1,893</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-desenvolver-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8914,6 +9649,11 @@
           <t>128,171</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-objetivo-pre-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8971,6 +9711,11 @@
           <t>1.445,497</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-oab-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9028,6 +9773,11 @@
           <t>13,796</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-relacionamento-ideal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9085,6 +9835,11 @@
           <t>2.137,571</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-executivo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9142,6 +9897,11 @@
           <t>66,296</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-performance-imab-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9199,6 +9959,11 @@
           <t>954,612</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-fifinvestidor-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9256,6 +10021,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-absolute-creta-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9313,6 +10083,11 @@
           <t>194,710</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-plus-quali-rf-credi-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9370,6 +10145,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-expert-sulamerica-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9427,6 +10207,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-arx-ipca-deb-incentivadas-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9484,6 +10269,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-vox-desenv-sustentavel-is-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9541,6 +10331,11 @@
           <t>34,940</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/inflacao-private-2027-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9598,6 +10393,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/expert-rb-asset-cdi-deb-incentivadas-fic-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9655,6 +10455,11 @@
           <t>2.894,171</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-expertise-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9712,6 +10517,11 @@
           <t>866,715</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/qualificado-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9769,6 +10579,11 @@
           <t>19,483</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-selecao-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9826,6 +10641,11 @@
           <t>133,651</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-renda-fixa-ativa/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9883,6 +10703,11 @@
           <t>313,138</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/indexa-tesouro-selic-fic-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9940,6 +10765,11 @@
           <t>3.103,041</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-personal-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9997,6 +10827,11 @@
           <t>125,908</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-supremo-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10054,6 +10889,11 @@
           <t>149,794</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-unique-rf-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10111,6 +10951,11 @@
           <t>2.398,591</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-especial-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10168,6 +11013,11 @@
           <t>14.155,221</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fic-maxi-renda-fixa-cred-priv/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10225,6 +11075,11 @@
           <t>531,259</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fidelidade-private-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10280,6 +11135,11 @@
       <c r="K39" t="inlineStr">
         <is>
           <t>1.293,248</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa/fidelidade-ii-rf-cred-priv/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -10294,7 +11154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10310,7 +11170,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -10325,12 +11185,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -10345,12 +11205,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -10410,6 +11275,11 @@
           <t>153,838</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-beta-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10467,6 +11337,11 @@
           <t>5.163,293</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-giro-imediato-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10524,6 +11399,11 @@
           <t>47,704</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-omega-ref-di-rf/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10581,6 +11461,11 @@
           <t>2.048,258</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-pleno-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10638,6 +11523,11 @@
           <t>872,706</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-preferencial-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10695,6 +11585,11 @@
           <t>13.911,673</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-sigma-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10752,6 +11647,11 @@
           <t>9.604,168</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-rubi-rf-ref-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10809,6 +11709,11 @@
           <t>18.273,507</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-mega-rf-referenc-di/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10864,6 +11769,11 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>10.092,191</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-referenciado/fic-top-private-rf-ref-di/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -10878,7 +11788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10894,7 +11804,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -10909,12 +11819,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -10929,12 +11839,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -10992,6 +11907,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>237,414</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/renda-fixa-curto-prazo/fic-renda-fixa/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -11006,7 +11926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11022,7 +11942,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -11037,12 +11957,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -11057,12 +11977,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -11122,6 +12047,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-cred-priv-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11179,6 +12109,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-multigestor-global-equit-s/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11236,6 +12171,11 @@
           <t>2.039,830</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-bolsa-americana-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11293,6 +12233,11 @@
           <t>21,113</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-juros-e-moedas-mm-plus/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11350,6 +12295,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-funcionarios-estrategia-livre-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11407,6 +12357,11 @@
           <t>540,034</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/multimercado-rv-30/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11464,6 +12419,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-estrategia-livre-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11521,6 +12481,11 @@
           <t>8,878</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-short-dolar-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11578,6 +12543,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-long-short/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11635,6 +12605,11 @@
           <t>2,907</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11692,6 +12667,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-long-bias-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11749,6 +12729,11 @@
           <t>2,386</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-euro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11806,6 +12791,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-estrategico-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -11863,6 +12853,11 @@
           <t>501,310</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/indexa-ouro-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11920,6 +12915,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fof-smart-mult-strategia-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11977,6 +12977,11 @@
           <t>37,650</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-hedge-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12034,6 +13039,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/hashdex-nasdaq-crypto-index-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12091,6 +13101,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/capital-protegido-ciclico-iii-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12148,6 +13163,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/capital-protegido-ibovespa-ciclico-i-fic-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -12205,6 +13225,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-fim-capital-protegido-ciclico-ii/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12262,6 +13287,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-capital-protegido-cesta-agro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12319,6 +13349,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-expert-spx-nimitz-multimercado/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -12376,6 +13411,11 @@
           <t>891,384</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-alocacao-macro-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12433,6 +13473,11 @@
           <t>799,440</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-juros-e-moedas-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -12490,6 +13535,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-caixa-expert-btg-pactual-x10-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -12547,6 +13597,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/fic-expert-pimco-income-mm/Paginas/default.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12602,6 +13657,11 @@
       <c r="K28" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/multimercado/expert-giant-zarathustra-fic-multimercado/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -12616,7 +13676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12632,7 +13692,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -12647,12 +13707,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -12667,12 +13727,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -12730,6 +13795,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>83,873</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/cambial/fic-indexa-dolar-cambial/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -12744,7 +13814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12760,7 +13830,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -12775,12 +13845,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -12795,19 +13865,24 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12858,13 +13933,18 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>302,922</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-dividendos/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12915,13 +13995,18 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>11,995</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-efundos-ibovespa/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12972,13 +14057,18 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>9,700</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/atena-fic-acoes-funcionarios-livre-quant/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -13029,13 +14119,18 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>299,253</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-bdr-nivel-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -13086,13 +14181,18 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>489,187</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-small-caps-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -13143,13 +14243,18 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>78,102</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-consumo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -13200,13 +14305,18 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>2,671</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-sustentabilidade-empresarial-ise-is/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -13257,13 +14367,18 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>65,705</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras-plus/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -13314,13 +14429,18 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>84,277</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-ibovespa/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -13371,13 +14491,18 @@
       <c r="K11" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-multigestor/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13428,13 +14553,18 @@
       <c r="K12" t="inlineStr">
         <is>
           <t>147,465</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-construcao-civil/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13485,13 +14615,18 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>127,311</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-infraestrutura/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13542,13 +14677,18 @@
       <c r="K14" t="inlineStr">
         <is>
           <t>47,594</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/atena-fic-acoes-livre-quant/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -13599,13 +14739,18 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>144,951</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras-presal/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -13656,13 +14801,18 @@
       <c r="K16" t="inlineStr">
         <is>
           <t>50,924</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-banco-do-brasil-plus/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -13713,13 +14863,18 @@
       <c r="K17" t="inlineStr">
         <is>
           <t>572,055</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-vale-do-rio-doce/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -13770,13 +14925,18 @@
       <c r="K18" t="inlineStr">
         <is>
           <t>413,157</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-seguridade/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -13827,13 +14987,18 @@
       <c r="K19" t="inlineStr">
         <is>
           <t>21,063</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-ibrx-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -13884,13 +15049,18 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>31,693</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-setor-financeiro/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -13941,13 +15111,18 @@
       <c r="K21" t="inlineStr">
         <is>
           <t>2,316</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-dividendos-quantitativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -13998,13 +15173,18 @@
       <c r="K22" t="inlineStr">
         <is>
           <t>41,189</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-pibb-ibrx-50/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -14055,13 +15235,18 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>34,936</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-ibovespa-ativo/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -14112,13 +15297,18 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>764,909</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-petrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -14169,13 +15359,18 @@
       <c r="K25" t="inlineStr">
         <is>
           <t>4,027</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-indexa-iagro/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -14226,13 +15421,18 @@
       <c r="K26" t="inlineStr">
         <is>
           <t>4,875</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-compromisso-bdr-nivel-i/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -14283,13 +15483,18 @@
       <c r="K27" t="inlineStr">
         <is>
           <t>20,989</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/seguridade-ii-acoes/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -14340,13 +15545,18 @@
       <c r="K28" t="inlineStr">
         <is>
           <t>238,332</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/acoes-eletrobras/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -14397,13 +15607,18 @@
       <c r="K29" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/fic-acoes-expert-verde-am-long-bias/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AÇÕES</t>
+          <t>ACOES</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -14454,6 +15669,11 @@
       <c r="K30" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/acoes/expert-claritas-valor-fic-acoes/Paginas/default.aspx</t>
         </is>
       </c>
     </row>
@@ -14468,7 +15688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14484,7 +15704,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Data Início</t>
+          <t>Data Inicio</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -14499,12 +15719,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Variação Dia (%)</t>
+          <t>Variacao Dia (%)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acum. Mês (%)</t>
+          <t>Acum. Mes (%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -14519,19 +15739,24 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PL (milhões R$)</t>
+          <t>PL (milhoes R$)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PL Médio (milhões R$)</t>
+          <t>PL Medio (milhoes R$)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FUNDO DE ÍNDICE</t>
+          <t>FUNDO DE INDICE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14582,6 +15807,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>41,204</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.caixa.gov.br/fundos-investimento/fundo-de-indice/etf-ibovespa-fundo-de-indice/Paginas/default.aspx</t>
         </is>
       </c>
     </row>

</xml_diff>